<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-10-23.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-10-23.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-10-23.xlsx
@@ -1353,6 +1353,9 @@
       <c r="C111" t="str">
         <v>286_红蕾丝_undefined_Rosa rugosa Thunb._10stems</v>
       </c>
+      <c r="F111" t="str">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -1411,7 +1414,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0991010125156173681061025759786551055105305555510555315131253455101510655510551086105510108561010651051266101055510105510151553151010101010202015202155105100</v>
+        <v>09910101251561736810610257597865510551053055555105553151312534551015106555105510861055101085610106510512661010555101055101515531510101010102020152021551051010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>